<commit_message>
Expand June 6-13 set: 7 deals across 6 sectors; $25M raise floor
Raise floor raised to >$25M (drop Vinyl Equity $20M). Add Current ($80M,
Banking & Lending), Octus/LevPro (Capital Markets M&A), Nuvei/Payoneer
($2.75B Payments M&A, agreement dated Jun 12). Financial Info & Analytics
and Corporate Financial Function have no qualifying in-window deal.
</commit_message>
<xml_diff>
--- a/fintech-deals-2026-06-06_06-13.xlsx
+++ b/fintech-deals-2026-06-06_06-13.xlsx
@@ -12,7 +12,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Growth Raises'!$A$1:$K$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Acquisitions'!$A$1:$K$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Acquisitions'!$A$1:$K$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -453,8 +453,8 @@
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
@@ -533,40 +533,42 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Vinyl Equity</t>
+          <t>Digital Asset</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Jump Capital</t>
+          <t>a16z crypto</t>
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="G2" s="2" t="inlineStr"/>
+        <v>355</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>2000</v>
+      </c>
       <c r="H2" s="2" t="inlineStr"/>
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>A US capital-markets infrastructure provider and SEC-registered transfer agent.</t>
+          <t>A US developer of the Canton Network blockchain for institutional capital markets.</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/vinyl-equity-raises-20-million-led-by-jump-capital-as-its-infrastructure-powers-modern-capital-markets-and-corporate-transactions-302795321.html</t>
+          <t>https://www.prnewswire.com/news-releases/digital-asset-raises-355-million-to-accelerate-cantons-role-as-onchain-infrastructure-for-capital-markets-302797427.html</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Capital Markets Tech</t>
+          <t>Banking &amp; Lending Tech</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -576,35 +578,35 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Digital Asset</t>
+          <t>Current</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>a16z crypto</t>
+          <t>Springcoast Partners</t>
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>355</v>
+        <v>80</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="H3" s="2" t="inlineStr"/>
       <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>A US developer of the Canton Network blockchain for institutional capital markets.</t>
+          <t>A US consumer neobank offering banking, spending and credit-building products.</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/digital-asset-raises-355-million-to-accelerate-cantons-role-as-onchain-infrastructure-for-capital-markets-302797427.html</t>
+          <t>https://www.thebankslate.com/2026/06/neobank-current-raises-80-million-in-latest-funding-round/</t>
         </is>
       </c>
     </row>
@@ -665,15 +667,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
@@ -786,7 +788,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Real Estate &amp; Mortgage Tech</t>
+          <t>Capital Markets Tech</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -801,37 +803,129 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Kiavi</t>
+          <t>LevPro</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Figure</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="n">
-        <v>717</v>
-      </c>
+          <t>Octus</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr"/>
       <c r="H3" s="2" t="inlineStr"/>
       <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="2" t="inlineStr">
         <is>
+          <t>A US front-office software provider for CLO and private-credit portfolio management and trading.</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>https://octus.com/company/news/octus-signs-definitive-agreement-to-acquire-levpro/</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Real Estate &amp; Mortgage Tech</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Strategic M&amp;A</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Kiavi</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Figure</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>717</v>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
           <t>A US AI-powered lending platform for residential real-estate investors.</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>https://www.kiavi.com/press/figure-acquires-kiavi</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Payments</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Strategic M&amp;A</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Payoneer</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Nuvei</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>2750</v>
+      </c>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>A US-based global cross-border payments and money-movement platform for SMBs.</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/nuvei-to-acquire-payoneer-for-2-75-billion-creating-a-leading-global-platform-for-local-and-cross-border-commerce-302800166.html</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K3"/>
+  <autoFilter ref="A1:K5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add EDGE Markets and nesto from subagent sweep (June 6-13)
Swarm mostly rate-limited but two agents completed: EDGE Markets ($29.2M
Series A, Payments, Jun 8) and nesto (~$220M Series E, Real Estate &
Mortgage, Jun 10) - latter independently confirmed by two agents. Now 9
deals across 6 sectors; Financial Info & Analytics and Corporate Financial
Function remain empty for the week.
</commit_message>
<xml_diff>
--- a/fintech-deals-2026-06-06_06-13.xlsx
+++ b/fintech-deals-2026-06-06_06-13.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Acquisitions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Growth Raises'!$A$1:$K$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Growth Raises'!$A$1:$K$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Acquisitions'!$A$1:$K$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -655,8 +655,96 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Payments</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>EDGE Markets</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>CoinFund</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>29.2</v>
+      </c>
+      <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>A US developer of payment-rail and settlement infrastructure for prediction markets and regulated gaming.</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/edge-markets-raises-29-2-million-series-a-funding-round-302793671.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Real Estate &amp; Mortgage Tech</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>nesto</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>La Caisse</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>220</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>1070</v>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>A Canadian mortgage technology and financing platform with white-label cloud and AI software for lenders.</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.globenewswire.com/news-release/2026/06/10/3309762/0/en/nesto-raises-302-million-Series-E-at-1-47-billion-valuation-to-accelerate-growth.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K4"/>
+  <autoFilter ref="A1:K6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add Adyen/Orb (Corporate Financial Function) from deep agent sweep
Adyen acquires Orb ($335M, billing/revenue-mgmt, 11 Jun) fills the
Corporate Financial Function gap. Now 10 deals across 7 of 8 sectors.
Financial Info & Analytics remains the sole empty sector - exhaustively
verified (only in-window F&A rounds, Capsa AI $18M and Vinyl Equity $20M,
are below the $25M floor).
</commit_message>
<xml_diff>
--- a/fintech-deals-2026-06-06_06-13.xlsx
+++ b/fintech-deals-2026-06-06_06-13.xlsx
@@ -12,7 +12,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Growth Raises'!$A$1:$K$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Acquisitions'!$A$1:$K$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Acquisitions'!$A$1:$K$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -755,7 +755,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1012,8 +1012,55 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Corporate Financial Function</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Strategic M&amp;A</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Orb</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Adyen</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>335</v>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>A US enterprise billing and revenue-management platform for usage-based pricing.</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adyen.com/press-and-media/jtrg4qd7j3p4rj</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K5"/>
+  <autoFilter ref="A1:K6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Complete June 6-13: 14 deals across all 8 sectors
Fill Financial Info & Analytics gap (Hypha $50M raise; Blockworks/Messari
and K2 Integrity/RiskFront AI M&A) and add second Corporate Financial
Function deal (Salesforce/m3ter). All 8 sectors now covered; every deal
date-verified against a primary source via the agent swarm + main-thread
checks.
</commit_message>
<xml_diff>
--- a/fintech-deals-2026-06-06_06-13.xlsx
+++ b/fintech-deals-2026-06-06_06-13.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Acquisitions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Growth Raises'!$A$1:$K$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Acquisitions'!$A$1:$K$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Growth Raises'!$A$1:$K$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Acquisitions'!$A$1:$K$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -743,8 +743,51 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Financial Info &amp; Analytics</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Hypha</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>TriEdge Investments</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>A US AI-native investment-intelligence platform structuring data across private credit and private equity.</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.businesswire.com/news/home/20260611628926/en/Hypha-Emerges-From-Stealth-Announces-a-$50M-Seed-Round</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K6"/>
+  <autoFilter ref="A1:K7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -755,7 +798,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1059,8 +1102,145 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Corporate Financial Function</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Strategic M&amp;A</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>m3ter</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Salesforce</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>A UK usage-based billing and revenue-metering platform for software companies.</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.salesforce.com/news/stories/salesforce-signs-definitive-agreement-to-acquire-m3ter/</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Financial Info &amp; Analytics</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Strategic M&amp;A</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Messari</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Blockworks</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>A US crypto market-data, research and intelligence platform.</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.businesswire.com/news/home/20260611031601/en/Blockworks-Acquires-Messari-Combining-the-Two-Largest-Crypto-Data-Platforms</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Financial Info &amp; Analytics</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Strategic M&amp;A</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>RiskFront AI</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>K2 Integrity</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>A US developer of agentic AI for financial-crime (AML) compliance and risk operations.</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>https://fintech.global/2026/06/10/k2-integrity-targets-financial-crime-with-ai-deal/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K6"/>
+  <autoFilter ref="A1:K9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add KOHO (Banking & Lending) from weekly-list extraction
KOHO C$130M (~$95M) Series E at unicorn valuation, led by Mubadala,
11 Jun - Canadian neobank. Now 15 deals across 8 sectors. Diagnosis of
under-counting (403-blocked sources, M&A blind spot) addressed via new
method-based agent swarm now running.
</commit_message>
<xml_diff>
--- a/fintech-deals-2026-06-06_06-13.xlsx
+++ b/fintech-deals-2026-06-06_06-13.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Acquisitions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Growth Raises'!$A$1:$K$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Growth Raises'!$A$1:$K$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Acquisitions'!$A$1:$K$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -786,8 +786,53 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Banking &amp; Lending Tech</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>KOHO</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Mubadala</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>95</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>970</v>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>A Canadian consumer neobank offering spending, savings and credit-building products.</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>https://betakit.com/koho-becomes-canadas-latest-unicorn-following-130-million-series-e-round/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K7"/>
+  <autoFilter ref="A1:K8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add Morpho ($175M DeFi lending) - final June 6-13 tally: 16 deals
Method-based swarm (press-wire, acquirer-enum, PE/vertical, regional,
funding-tracker) added KOHO and Morpho; M&A side exhaustively confirmed
with no new acquisitions. Excluded Climate First Bancorp (chartered bank,
not tech). 16 deals across all 8 sectors.
</commit_message>
<xml_diff>
--- a/fintech-deals-2026-06-06_06-13.xlsx
+++ b/fintech-deals-2026-06-06_06-13.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Acquisitions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Growth Raises'!$A$1:$K$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Growth Raises'!$A$1:$K$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Acquisitions'!$A$1:$K$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -831,8 +831,53 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Banking &amp; Lending Tech</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Paradigm, a16z crypto, Ribbit Capital</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>175</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>2000</v>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>A DeFi lending protocol building an open, onchain credit network used by crypto institutions.</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>https://fortune.com/2026/06/09/morpho-fundraise-a16z-crypto-paradigm-ribbit-capital-175-million/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K8"/>
+  <autoFilter ref="A1:K9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>